<commit_message>
halfway done with win 10 module vulnID updates
</commit_message>
<xml_diff>
--- a/Scanning Scripts/_workstations/Batch Execution/Summary - 5-21-2020_124812.xlsx
+++ b/Scanning Scripts/_workstations/Batch Execution/Summary - 5-21-2020_124812.xlsx
@@ -5,23 +5,24 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\bdsca7swan200\BDSC_share\Information Assurance\STIG\Scripts\Scanning Scripts\_workstations\Batch Execution\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brad\Documents\github\STIG\Scanning Scripts\_workstations\Batch Execution\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12450"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="3" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
-    <sheet name="Summary - 5-21-2020_124812" sheetId="1" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
+    <sheet name="Summary - 5-21-2020_124812" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14939" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15051" uniqueCount="190">
   <si>
     <t xml:space="preserve">Computer         </t>
   </si>
@@ -589,6 +590,9 @@
   <si>
     <t>BDSCWKNAEAGCBAB</t>
   </si>
+  <si>
+    <t>V-77223</t>
+  </si>
 </sst>
 </file>
 
@@ -1101,15 +1105,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -1402,463 +1398,282 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:B58"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>124</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>111</v>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>0</v>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>100</v>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>1</v>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>6</v>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>4</v>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>0</v>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>6</v>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>2</v>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>112</v>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>4</v>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>6</v>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>4</v>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>189</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>2</v>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>1</v>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>4</v>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <v>4</v>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>4</v>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>4</v>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29">
-        <v>4</v>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30">
-        <v>5</v>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31">
-        <v>1</v>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32">
-        <v>0</v>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
-      <c r="B33">
-        <v>5</v>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>51</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34">
-        <v>0</v>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>52</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35">
-        <v>0</v>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36">
-        <v>0</v>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37">
-        <v>3</v>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>37</v>
-      </c>
-      <c r="B38">
-        <v>4</v>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>40</v>
-      </c>
-      <c r="B41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>41</v>
-      </c>
-      <c r="B42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>42</v>
-      </c>
-      <c r="B43">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>45</v>
-      </c>
-      <c r="B46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>46</v>
-      </c>
-      <c r="B47">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>47</v>
-      </c>
-      <c r="B48">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>48</v>
-      </c>
-      <c r="B49">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>49</v>
-      </c>
-      <c r="B50">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>50</v>
-      </c>
-      <c r="B51">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>51</v>
-      </c>
-      <c r="B52">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>52</v>
-      </c>
-      <c r="B53">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>53</v>
-      </c>
-      <c r="B54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>54</v>
-      </c>
-      <c r="B55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>55</v>
-      </c>
-      <c r="B56">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>56</v>
-      </c>
-      <c r="B57">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
         <v>57</v>
-      </c>
-      <c r="B58">
-        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1867,6 +1682,685 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:C79"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>4</v>
+      </c>
+      <c r="C27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>5</v>
+      </c>
+      <c r="C33" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>3</v>
+      </c>
+      <c r="C37" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>0</v>
+      </c>
+      <c r="C40" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>0</v>
+      </c>
+      <c r="C41" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>0</v>
+      </c>
+      <c r="C42" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>4</v>
+      </c>
+      <c r="C43" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>4</v>
+      </c>
+      <c r="C44" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>0</v>
+      </c>
+      <c r="C45" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>0</v>
+      </c>
+      <c r="C46" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>64</v>
+      </c>
+      <c r="C48" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+      <c r="C49" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>4</v>
+      </c>
+      <c r="C52" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>0</v>
+      </c>
+      <c r="C54" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>0</v>
+      </c>
+      <c r="C55" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>3</v>
+      </c>
+      <c r="C56" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>96</v>
+      </c>
+      <c r="C57" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>124</v>
+      </c>
+      <c r="C58" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C59" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C60" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C61" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C62" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C63" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C64" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C65" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="66" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C66" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C67" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="68" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C68" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="69" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C69" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="70" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="71" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C71" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="72" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C72" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="73" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C73" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="74" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C74" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="75" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C75" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="76" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C76" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="77" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C77" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="78" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C78" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="79" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C79" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BF132"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -24952,7 +25446,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BF129"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -47462,7 +47956,7 @@
         <v>124</v>
       </c>
       <c r="C129">
-        <f t="shared" ref="C129:BF131" si="0">COUNTIF(C1:C128,"Fail")</f>
+        <f t="shared" ref="C129:BF129" si="0">COUNTIF(C1:C128,"Fail")</f>
         <v>4</v>
       </c>
       <c r="D129">
@@ -47688,7 +48182,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:BF128">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",A2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>